<commit_message>
Save state before refactoring
</commit_message>
<xml_diff>
--- a/database/event/event_scores_lookup.xlsx
+++ b/database/event/event_scores_lookup.xlsx
@@ -425,10 +425,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>event_name</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>event_score</t>
@@ -438,241 +443,101 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>blast-bounty-2025-season-1</t>
+          <t>blast-bounty-2026-season-1-finals</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.7451807228915663</v>
+        <v>0.3846526851739605</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>iem-katowice-2025</t>
+          <t>iem-krakw-2026</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.0556</v>
+        <v>0.6222532263690269</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>pgl-cluj-napoca-2025</t>
+          <t>pgl-cluj-napoca-2026</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5252</v>
+        <v>0.6018529241459177</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>esl-pro-league-season-21</t>
+          <t>EPL-S23</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.0866</v>
+        <v>0.443489932885906</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>blast-open-lisbon-2025</t>
+          <t>blast-open-rotterdam-2026</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.204670050761422</v>
+        <v>0.5915355531162337</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>pgl-bucharest-2025</t>
+          <t>pgl-bucharest-2026</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5455301455301456</v>
+        <v>0.2200135226504395</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>iem-melbourne-2025</t>
+          <t>iem-rio-2026</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.8994</v>
+        <v>0.452928870292887</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>blast-rivals-2025-season-1</t>
+          <t>blast-rivals-2026-season-1</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.5978</v>
+        <v>0.3300948144679855</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>pgl-astana-2025</t>
+          <t>pgl-astana-2026</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.5206</v>
+        <v>0.3545303408146301</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>iem-dallas-2025</t>
+          <t>iem-atlanta-2026</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.7856</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>blasttv-austin-major-2025</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.868</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>fissure-playground-1</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.282</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>iem-cologne-2025</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0.888</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>blast-bounty-2025-season-2</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.7164</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>esports-world-cup-2025</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1.119491525423729</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>blast-open-london-2025</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0.8907987866531852</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>fissure-playground-2</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>0.7642</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>esl-pro-league-season-22</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1.278348214285714</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>cs-asia-championships-2025</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>0.34</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>thunderpick-world-championship-2025</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>0.427578947368421</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>pgl-masters-bucharest-2025</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>0.4148148148148148</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>iem-chengdu-2025</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1.273015873015873</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>blast-rivals-2025-season-2</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>0.7689217758985201</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>starladder-budapest-major-2025</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1.166025641025641</v>
+        <v>0.3750172532781229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>